<commit_message>
add QuickSilver driver box replacement manual
</commit_message>
<xml_diff>
--- a/Magnetometer_Operations/Forms/thermal_demag_sheet.xlsx
+++ b/Magnetometer_Operations/Forms/thermal_demag_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10808"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yimingzhang/Desktop/Github/anorthosite_xenoliths/Data/SAM files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yimingzhang/Github/lab_protocols/Magnetometer_Operations/Forms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AEF14D-B5E1-0E43-A1BC-F0AB67F4BD2F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA68152-9197-714C-A256-05B809346C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="1380" windowWidth="28040" windowHeight="16620" xr2:uid="{E1B9C4B8-376C-6D4E-873B-881E0D0CAFD2}"/>
+    <workbookView xWindow="5620" yWindow="1120" windowWidth="28040" windowHeight="16620" xr2:uid="{E1B9C4B8-376C-6D4E-873B-881E0D0CAFD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="9">
   <si>
     <t>temp</t>
   </si>
@@ -442,17 +442,16 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="11" width="5.83203125" style="1" customWidth="1"/>
-    <col min="12" max="14" width="5.83203125" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="10.83203125" style="1"/>
+    <col min="3" max="8" width="5.83203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -465,14 +464,8 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3" t="s">
@@ -493,26 +486,8 @@
       <c r="H2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -523,14 +498,8 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-    </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -541,14 +510,8 @@
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
         <v>4</v>
@@ -559,14 +522,8 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
@@ -577,14 +534,8 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
       <c r="B7" s="3" t="s">
         <v>4</v>
@@ -595,14 +546,8 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="B8" s="3" t="s">
         <v>3</v>
@@ -613,14 +558,8 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="B9" s="3" t="s">
         <v>4</v>
@@ -631,14 +570,8 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="3" t="s">
         <v>3</v>
@@ -649,14 +582,8 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="3" t="s">
         <v>4</v>
@@ -667,14 +594,8 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3" t="s">
         <v>3</v>
@@ -685,14 +606,8 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="s">
         <v>4</v>
@@ -703,14 +618,8 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="3" t="s">
         <v>3</v>
@@ -721,14 +630,8 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="s">
         <v>4</v>
@@ -739,14 +642,8 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="s">
         <v>3</v>
@@ -757,14 +654,8 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="s">
         <v>4</v>
@@ -775,14 +666,8 @@
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="s">
         <v>3</v>
@@ -793,14 +678,8 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="s">
         <v>4</v>
@@ -811,14 +690,8 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="s">
         <v>3</v>
@@ -829,14 +702,8 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>4</v>
@@ -847,14 +714,8 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>3</v>
@@ -865,14 +726,8 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>4</v>
@@ -883,14 +738,8 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="s">
         <v>3</v>
@@ -901,14 +750,8 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="3" t="s">
         <v>4</v>
@@ -919,14 +762,8 @@
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="3" t="s">
         <v>3</v>
@@ -937,14 +774,8 @@
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3" t="s">
         <v>4</v>
@@ -955,14 +786,8 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
         <v>3</v>
@@ -973,14 +798,8 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="3" t="s">
         <v>4</v>
@@ -991,14 +810,8 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>3</v>
@@ -1009,14 +822,8 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
-      <c r="M30" s="3"/>
-      <c r="N30" s="3"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>4</v>
@@ -1027,14 +834,8 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>3</v>
@@ -1045,14 +846,8 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>4</v>
@@ -1063,14 +858,8 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
-    </row>
-    <row r="34" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
       <c r="B34" s="3" t="s">
         <v>3</v>
@@ -1081,14 +870,8 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-    </row>
-    <row r="35" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
         <v>4</v>
@@ -1099,14 +882,8 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
-      <c r="N35" s="3"/>
-    </row>
-    <row r="36" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
         <v>3</v>
@@ -1117,14 +894,8 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
-      <c r="N36" s="3"/>
-    </row>
-    <row r="37" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="B37" s="3" t="s">
         <v>4</v>
@@ -1135,14 +906,8 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
-      <c r="N37" s="3"/>
-    </row>
-    <row r="38" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
       <c r="B38" s="3" t="s">
         <v>3</v>
@@ -1153,14 +918,8 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
-      <c r="N38" s="3"/>
-    </row>
-    <row r="39" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
       <c r="B39" s="3" t="s">
         <v>4</v>
@@ -1171,14 +930,8 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
-    </row>
-    <row r="40" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
       <c r="B40" s="3" t="s">
         <v>3</v>
@@ -1189,14 +942,8 @@
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
-      <c r="N40" s="3"/>
-    </row>
-    <row r="41" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
       <c r="B41" s="3" t="s">
         <v>4</v>
@@ -1207,14 +954,8 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
-      <c r="N41" s="3"/>
-    </row>
-    <row r="42" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
         <v>3</v>
@@ -1225,14 +966,8 @@
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-      <c r="N42" s="3"/>
-    </row>
-    <row r="43" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
         <v>4</v>
@@ -1243,14 +978,8 @@
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-      <c r="N43" s="3"/>
-    </row>
-    <row r="44" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3" t="s">
         <v>3</v>
@@ -1261,14 +990,8 @@
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
-      <c r="N44" s="3"/>
-    </row>
-    <row r="45" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="B45" s="3" t="s">
         <v>4</v>
@@ -1279,22 +1002,14 @@
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
-      <c r="K45" s="3"/>
-      <c r="L45" s="3"/>
-      <c r="M45" s="3"/>
-      <c r="N45" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
   </mergeCells>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="2"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="20"/>
 </worksheet>
 </file>
</xml_diff>